<commit_message>
Test batch 4: revised own estimates and programme causes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-reports/batch4/batch4-input-vs-output.xlsx
+++ b/test-reports/batch4/batch4-input-vs-output.xlsx
@@ -4,9 +4,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Input vs output" sheetId="1" r:id="rId1"/>
+    <sheet name="Why programmes are long" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Input vs output'!$A$1:$Z$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Input vs output'!$A$1:$AA$31</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -400,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z31"/>
+  <dimension ref="A1:AA31"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -421,13 +422,14 @@
     <col min="17" max="17" width="24.83203125" customWidth="1"/>
     <col min="18" max="18" width="20.83203125" customWidth="1"/>
     <col min="19" max="19" width="24.83203125" customWidth="1"/>
-    <col min="20" max="20" width="12.83203125" customWidth="1"/>
-    <col min="21" max="21" width="16.83203125" customWidth="1"/>
-    <col min="22" max="22" width="12.83203125" customWidth="1"/>
-    <col min="23" max="23" width="24.83203125" customWidth="1"/>
-    <col min="24" max="24" width="15.83203125" customWidth="1"/>
-    <col min="25" max="25" width="45.83203125" customWidth="1"/>
-    <col min="26" max="26" width="60.83203125" customWidth="1"/>
+    <col min="20" max="20" width="24.83203125" customWidth="1"/>
+    <col min="21" max="21" width="12.83203125" customWidth="1"/>
+    <col min="22" max="22" width="16.83203125" customWidth="1"/>
+    <col min="23" max="23" width="12.83203125" customWidth="1"/>
+    <col min="24" max="24" width="24.83203125" customWidth="1"/>
+    <col min="25" max="25" width="15.83203125" customWidth="1"/>
+    <col min="26" max="26" width="45.83203125" customWidth="1"/>
+    <col min="27" max="27" width="60.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -489,24 +491,27 @@
         <v>Projento programme weeks</v>
       </c>
       <c r="T1" t="str">
+        <v>Programme diff % (mid)</v>
+      </c>
+      <c r="U1" t="str">
         <v>Confidence</v>
       </c>
-      <c r="U1" t="str">
+      <c r="V1" t="str">
         <v>Budget verdict</v>
       </c>
-      <c r="V1" t="str">
+      <c r="W1" t="str">
         <v>Risk level</v>
       </c>
-      <c r="W1" t="str">
+      <c r="X1" t="str">
         <v>Procurement (preferred)</v>
       </c>
-      <c r="X1" t="str">
+      <c r="Y1" t="str">
         <v>Report status</v>
       </c>
-      <c r="Y1" t="str">
+      <c r="Z1" t="str">
         <v>Report link</v>
       </c>
-      <c r="Z1" t="str">
+      <c r="AA1" t="str">
         <v>What needs changing</v>
       </c>
     </row>
@@ -563,31 +568,34 @@
         <v>43</v>
       </c>
       <c r="R2" t="str">
-        <v>95–120</v>
+        <v>80–90</v>
       </c>
       <c r="S2">
         <v>89</v>
       </c>
-      <c r="T2" t="str">
+      <c r="T2">
+        <v>5</v>
+      </c>
+      <c r="U2" t="str">
         <v>B</v>
       </c>
-      <c r="U2" t="str">
+      <c r="V2" t="str">
         <v>insufficient</v>
       </c>
-      <c r="V2" t="str">
+      <c r="W2" t="str">
         <v>Low</v>
       </c>
-      <c r="W2" t="str">
+      <c r="X2" t="str">
         <v>Traditional</v>
       </c>
-      <c r="X2" t="str">
+      <c r="Y2" t="str">
         <v>complete</v>
       </c>
-      <c r="Y2" t="str">
+      <c r="Z2" t="str">
         <v>https://www.projento.co.uk/report/96f932ad785446dc</v>
       </c>
-      <c r="Z2" t="str">
-        <v>Cost +18% on my mid (£2,906/m²) — check flat rates for a 3-storey block. Budget 'insufficient' is fair once fees/risk added.</v>
+      <c r="AA2" t="str">
+        <v>Programme OK. Cost +18% (£2,906/m²): check flat rates for a 3-storey block.</v>
       </c>
     </row>
     <row r="3">
@@ -637,37 +645,40 @@
         <v>-14</v>
       </c>
       <c r="P3" t="str">
-        <v>50–65</v>
+        <v>50–60</v>
       </c>
       <c r="Q3">
         <v>42</v>
       </c>
       <c r="R3" t="str">
-        <v>100–130</v>
+        <v>94–104</v>
       </c>
       <c r="S3">
         <v>112</v>
       </c>
-      <c r="T3" t="str">
+      <c r="T3">
+        <v>13</v>
+      </c>
+      <c r="U3" t="str">
         <v>C</v>
       </c>
-      <c r="U3" t="str">
+      <c r="V3" t="str">
         <v>none</v>
       </c>
-      <c r="V3" t="str">
+      <c r="W3" t="str">
         <v>High</v>
       </c>
-      <c r="W3" t="str">
+      <c r="X3" t="str">
         <v>Two-stage (PCSA)</v>
       </c>
-      <c r="X3" t="str">
+      <c r="Y3" t="str">
         <v>complete</v>
       </c>
-      <c r="Y3" t="str">
+      <c r="Z3" t="str">
         <v>https://www.projento.co.uk/report/e4106c1a0562476e</v>
       </c>
-      <c r="Z3" t="str">
-        <v>OK on cost. 42 weeks for 32 occupied flats looks short (I expected 50–65).</v>
+      <c r="AA3" t="str">
+        <v>Programme +13% (6 wks governance + 8 float); construction 42 wks short for 32 occupied flats (50–60). Cost OK.</v>
       </c>
     </row>
     <row r="4">
@@ -723,31 +734,34 @@
         <v>19</v>
       </c>
       <c r="R4" t="str">
-        <v>35–50</v>
+        <v>33–37</v>
       </c>
       <c r="S4">
         <v>62</v>
       </c>
-      <c r="T4" t="str">
+      <c r="T4">
+        <v>77</v>
+      </c>
+      <c r="U4" t="str">
         <v>B</v>
       </c>
-      <c r="U4" t="str">
+      <c r="V4" t="str">
         <v>tight</v>
       </c>
-      <c r="V4" t="str">
+      <c r="W4" t="str">
         <v>Low</v>
       </c>
-      <c r="W4" t="str">
+      <c r="X4" t="str">
         <v>Traditional</v>
       </c>
-      <c r="X4" t="str">
+      <c r="Y4" t="str">
         <v>complete</v>
       </c>
-      <c r="Y4" t="str">
+      <c r="Z4" t="str">
         <v>https://www.projento.co.uk/report/3301fe2084cf42e6</v>
       </c>
-      <c r="Z4" t="str">
-        <v>OK on cost. 19 weeks on site for parking and planting looks long (I expected 10–14).</v>
+      <c r="AA4" t="str">
+        <v>Programme +77%: 20 wks design and 12 wks tender for car park/landscaping (6+6 design, 6 tender). Construction 19 wks long (10–14).</v>
       </c>
     </row>
     <row r="5">
@@ -797,37 +811,40 @@
         <v>-6</v>
       </c>
       <c r="P5" t="str">
-        <v>70–85</v>
+        <v>65–80</v>
       </c>
       <c r="Q5">
         <v>80</v>
       </c>
       <c r="R5" t="str">
-        <v>120–145</v>
+        <v>120–140</v>
       </c>
       <c r="S5">
         <v>163</v>
       </c>
-      <c r="T5" t="str">
+      <c r="T5">
+        <v>25</v>
+      </c>
+      <c r="U5" t="str">
         <v>C</v>
       </c>
-      <c r="U5" t="str">
+      <c r="V5" t="str">
         <v>tight</v>
       </c>
-      <c r="V5" t="str">
+      <c r="W5" t="str">
         <v>Low</v>
       </c>
-      <c r="W5" t="str">
+      <c r="X5" t="str">
         <v>Two-stage (PCSA)</v>
       </c>
-      <c r="X5" t="str">
+      <c r="Y5" t="str">
         <v>complete</v>
       </c>
-      <c r="Y5" t="str">
+      <c r="Z5" t="str">
         <v>https://www.projento.co.uk/report/c617fd4759094df6</v>
       </c>
-      <c r="Z5" t="str">
-        <v>OK on cost and 80 weeks. Target date correctly flagged as missed (163 weeks, Gateway 2 18 weeks). No change.</v>
+      <c r="AA5" t="str">
+        <v>Programme +25%: 12 wks float + 4 gates on top of 18-wk BSR Gateway 2. Construction 80 wks at top of range. Target miss correctly flagged. Cost OK.</v>
       </c>
     </row>
     <row r="6">
@@ -859,22 +876,22 @@
         <v>£3,000k</v>
       </c>
       <c r="J6" t="str">
-        <v>£1,800k–£2,600k</v>
+        <v>£1,440k–£2,080k</v>
       </c>
       <c r="K6" t="str">
         <v>£1,211k</v>
       </c>
       <c r="L6">
-        <v>-45</v>
+        <v>-31</v>
       </c>
       <c r="M6" t="str">
-        <v>£2,600k–£3,800k</v>
+        <v>£2,100k–£3,000k</v>
       </c>
       <c r="N6" t="str">
         <v>£1,287k–£1,895k</v>
       </c>
       <c r="O6">
-        <v>-53</v>
+        <v>-41</v>
       </c>
       <c r="P6" t="str">
         <v>12–14</v>
@@ -883,31 +900,34 @@
         <v>14</v>
       </c>
       <c r="R6" t="str">
-        <v>30–40</v>
+        <v>40–42</v>
       </c>
       <c r="S6">
         <v>42</v>
       </c>
-      <c r="T6" t="str">
+      <c r="T6">
+        <v>2</v>
+      </c>
+      <c r="U6" t="str">
         <v>C</v>
       </c>
-      <c r="U6" t="str">
+      <c r="V6" t="str">
         <v>sufficient</v>
       </c>
-      <c r="V6" t="str">
+      <c r="W6" t="str">
         <v>Low</v>
       </c>
-      <c r="W6" t="str">
+      <c r="X6" t="str">
         <v>Two-stage (PCSA)</v>
       </c>
-      <c r="X6" t="str">
+      <c r="Y6" t="str">
         <v>complete</v>
       </c>
-      <c r="Y6" t="str">
+      <c r="Z6" t="str">
         <v>https://www.projento.co.uk/report/eb56dd9077bb4d28</v>
       </c>
-      <c r="Z6" t="str">
-        <v>Cost about 40% below me (£378/m²) — study-room refresh with kitchens and lighting looks under-priced. Summer window respected (14 weeks). Good.</v>
+      <c r="AA6" t="str">
+        <v>Programme OK (summer window respected). Cost −16% vs revised (£378/m²).</v>
       </c>
     </row>
     <row r="7">
@@ -957,37 +977,40 @@
         <v>-6</v>
       </c>
       <c r="P7" t="str">
-        <v>32–40</v>
+        <v>30–36</v>
       </c>
       <c r="Q7">
         <v>32</v>
       </c>
       <c r="R7" t="str">
-        <v>90–110</v>
+        <v>68–75</v>
       </c>
       <c r="S7">
         <v>81</v>
       </c>
-      <c r="T7" t="str">
+      <c r="T7">
+        <v>13</v>
+      </c>
+      <c r="U7" t="str">
         <v>D</v>
       </c>
-      <c r="U7" t="str">
+      <c r="V7" t="str">
         <v>none</v>
       </c>
-      <c r="V7" t="str">
+      <c r="W7" t="str">
         <v>High</v>
       </c>
-      <c r="W7" t="str">
+      <c r="X7" t="str">
         <v>Traditional</v>
       </c>
-      <c r="X7" t="str">
+      <c r="Y7" t="str">
         <v>complete</v>
       </c>
-      <c r="Y7" t="str">
+      <c r="Z7" t="str">
         <v>https://www.projento.co.uk/report/adebcb25d69c4deb</v>
       </c>
-      <c r="Z7" t="str">
-        <v>OK on cost and weeks. No change.</v>
+      <c r="AA7" t="str">
+        <v>Programme +13% (float 6, gates 6). Cost OK.</v>
       </c>
     </row>
     <row r="8">
@@ -1043,31 +1066,34 @@
         <v>23</v>
       </c>
       <c r="R8" t="str">
-        <v>26–36</v>
+        <v>26–30</v>
       </c>
       <c r="S8">
         <v>42</v>
       </c>
-      <c r="T8" t="str">
+      <c r="T8">
+        <v>50</v>
+      </c>
+      <c r="U8" t="str">
         <v>B</v>
       </c>
-      <c r="U8" t="str">
+      <c r="V8" t="str">
         <v>tight</v>
       </c>
-      <c r="V8" t="str">
+      <c r="W8" t="str">
         <v>Low</v>
       </c>
-      <c r="W8" t="str">
+      <c r="X8" t="str">
         <v>Design and build (single stage)</v>
       </c>
-      <c r="X8" t="str">
+      <c r="Y8" t="str">
         <v>complete</v>
       </c>
-      <c r="Y8" t="str">
+      <c r="Z8" t="str">
         <v>https://www.projento.co.uk/report/e06a5d30de8d4283</v>
       </c>
-      <c r="Z8" t="str">
-        <v>OK on cost. 23 weeks for a 1,200 m² Cat A floor looks long (I expected 12–16).</v>
+      <c r="AA8" t="str">
+        <v>Programme +50%: construction 23 wks for a 1,200 m² Cat A floor (12–16). Cost OK.</v>
       </c>
     </row>
     <row r="9">
@@ -1099,55 +1125,58 @@
         <v>£5,000k</v>
       </c>
       <c r="J9" t="str">
-        <v>£3,250k–£4,500k</v>
+        <v>£3,000k–£4,000k</v>
       </c>
       <c r="K9" t="str">
         <v>£2,684k</v>
       </c>
       <c r="L9">
-        <v>-31</v>
+        <v>-23</v>
       </c>
       <c r="M9" t="str">
-        <v>£4,100k–£5,600k</v>
+        <v>£3,750k–£5,000k</v>
       </c>
       <c r="N9" t="str">
         <v>£3,263k–£4,349k</v>
       </c>
       <c r="O9">
-        <v>-25</v>
+        <v>-17</v>
       </c>
       <c r="P9" t="str">
-        <v>36–45</v>
+        <v>36–42</v>
       </c>
       <c r="Q9">
         <v>32</v>
       </c>
       <c r="R9" t="str">
-        <v>70–90</v>
+        <v>72–81</v>
       </c>
       <c r="S9">
         <v>83</v>
       </c>
-      <c r="T9" t="str">
+      <c r="T9">
+        <v>8</v>
+      </c>
+      <c r="U9" t="str">
         <v>B</v>
       </c>
-      <c r="U9" t="str">
+      <c r="V9" t="str">
         <v>sufficient</v>
       </c>
-      <c r="V9" t="str">
+      <c r="W9" t="str">
         <v>Low</v>
       </c>
-      <c r="W9" t="str">
+      <c r="X9" t="str">
         <v>Traditional</v>
       </c>
-      <c r="X9" t="str">
+      <c r="Y9" t="str">
         <v>complete</v>
       </c>
-      <c r="Y9" t="str">
+      <c r="Z9" t="str">
         <v>https://www.projento.co.uk/report/1c49f3825a7e48ed</v>
       </c>
-      <c r="Z9" t="str">
-        <v>Cost about 30% below me (£1,074/m²) for a full services strip-back with lift — check full-systems refurb rates for offices.</v>
+      <c r="AA9" t="str">
+        <v>Programme OK. Cost −23% vs revised (£1,074/m² for full services + lift).</v>
       </c>
     </row>
     <row r="10">
@@ -1197,37 +1226,40 @@
         <v>7</v>
       </c>
       <c r="P10" t="str">
-        <v>36–44</v>
+        <v>36–40</v>
       </c>
       <c r="Q10">
         <v>39</v>
       </c>
       <c r="R10" t="str">
-        <v>90–110</v>
+        <v>73–77</v>
       </c>
       <c r="S10">
         <v>94</v>
       </c>
-      <c r="T10" t="str">
+      <c r="T10">
+        <v>25</v>
+      </c>
+      <c r="U10" t="str">
         <v>B</v>
       </c>
-      <c r="U10" t="str">
+      <c r="V10" t="str">
         <v>none</v>
       </c>
-      <c r="V10" t="str">
+      <c r="W10" t="str">
         <v>Low</v>
       </c>
-      <c r="W10" t="str">
+      <c r="X10" t="str">
         <v>Traditional</v>
       </c>
-      <c r="X10" t="str">
+      <c r="Y10" t="str">
         <v>complete</v>
       </c>
-      <c r="Y10" t="str">
+      <c r="Z10" t="str">
         <v>https://www.projento.co.uk/report/5e554c82a9254483</v>
       </c>
-      <c r="Z10" t="str">
-        <v>Cost +14% — acceptable. No change.</v>
+      <c r="AA10" t="str">
+        <v>Programme +25%: float 7, gates 6, tender 12 for a £2m job. Cost +14%, acceptable.</v>
       </c>
     </row>
     <row r="11">
@@ -1277,37 +1309,40 @@
         <v>23</v>
       </c>
       <c r="P11" t="str">
-        <v>26–32</v>
+        <v>20–26</v>
       </c>
       <c r="Q11">
         <v>15</v>
       </c>
       <c r="R11" t="str">
-        <v>80–95</v>
+        <v>50–56</v>
       </c>
       <c r="S11">
         <v>59</v>
       </c>
-      <c r="T11" t="str">
+      <c r="T11">
+        <v>11</v>
+      </c>
+      <c r="U11" t="str">
         <v>D</v>
       </c>
-      <c r="U11" t="str">
+      <c r="V11" t="str">
         <v>tight</v>
       </c>
-      <c r="V11" t="str">
+      <c r="W11" t="str">
         <v>High</v>
       </c>
-      <c r="W11" t="str">
+      <c r="X11" t="str">
         <v>Traditional</v>
       </c>
-      <c r="X11" t="str">
+      <c r="Y11" t="str">
         <v>complete</v>
       </c>
-      <c r="Y11" t="str">
+      <c r="Z11" t="str">
         <v>https://www.projento.co.uk/report/504b6a2814704e9e</v>
       </c>
-      <c r="Z11" t="str">
-        <v>OK on cost. 15 weeks on site for a classroom extension looks short (I expected 26–32).</v>
+      <c r="AA11" t="str">
+        <v>Programme +11% total but construction 15 wks too short for a classroom extension (20–26). Cost OK.</v>
       </c>
     </row>
     <row r="12">
@@ -1339,55 +1374,58 @@
         <v>£1,100k</v>
       </c>
       <c r="J12" t="str">
-        <v>£680k–£1,050k</v>
+        <v>£680k–£900k</v>
       </c>
       <c r="K12" t="str">
         <v>£438k</v>
       </c>
       <c r="L12">
-        <v>-49</v>
+        <v>-45</v>
       </c>
       <c r="M12" t="str">
-        <v>£900k–£1,400k</v>
+        <v>£900k–£1,200k</v>
       </c>
       <c r="N12" t="str">
         <v>£463k–£780k</v>
       </c>
       <c r="O12">
-        <v>-50</v>
+        <v>-45</v>
       </c>
       <c r="P12" t="str">
-        <v>10–14</v>
+        <v>50–70</v>
       </c>
       <c r="Q12">
         <v>73</v>
       </c>
       <c r="R12" t="str">
-        <v>40–70</v>
+        <v>70–90</v>
       </c>
       <c r="S12">
         <v>114</v>
       </c>
-      <c r="T12" t="str">
+      <c r="T12">
+        <v>43</v>
+      </c>
+      <c r="U12" t="str">
         <v>D</v>
       </c>
-      <c r="U12" t="str">
+      <c r="V12" t="str">
         <v>sufficient</v>
       </c>
-      <c r="V12" t="str">
+      <c r="W12" t="str">
         <v>Medium</v>
       </c>
-      <c r="W12" t="str">
+      <c r="X12" t="str">
         <v>Traditional</v>
       </c>
-      <c r="X12" t="str">
+      <c r="Y12" t="str">
         <v>complete</v>
       </c>
-      <c r="Y12" t="str">
+      <c r="Z12" t="str">
         <v>https://www.projento.co.uk/report/fb10d2cf8bd34c22</v>
       </c>
-      <c r="Z12" t="str">
-        <v>Cost about 50% below me (£292/m²) for windows, roof and wall insulation — check fabric-only rates. 73 weeks spread over holidays is right in principle.</v>
+      <c r="AA12" t="str">
+        <v>Programme +43%: holiday spread gives 73 wks on site (50–70 expected) plus 12 tender, 9 float. Cost −45% (£292/m² for windows, roof, wall insulation) — check fabric-only scope/rates.</v>
       </c>
     </row>
     <row r="13">
@@ -1443,31 +1481,34 @@
         <v>20</v>
       </c>
       <c r="R13" t="str">
-        <v>55–70</v>
+        <v>50–56</v>
       </c>
       <c r="S13">
         <v>64</v>
       </c>
-      <c r="T13" t="str">
+      <c r="T13">
+        <v>21</v>
+      </c>
+      <c r="U13" t="str">
         <v>C</v>
       </c>
-      <c r="U13" t="str">
+      <c r="V13" t="str">
         <v>tight</v>
       </c>
-      <c r="V13" t="str">
+      <c r="W13" t="str">
         <v>Low</v>
       </c>
-      <c r="W13" t="str">
+      <c r="X13" t="str">
         <v>Traditional</v>
       </c>
-      <c r="X13" t="str">
+      <c r="Y13" t="str">
         <v>complete</v>
       </c>
-      <c r="Y13" t="str">
+      <c r="Z13" t="str">
         <v>https://www.projento.co.uk/report/abe0970ea3a040c8</v>
       </c>
-      <c r="Z13" t="str">
-        <v>OK on cost and weeks. No change.</v>
+      <c r="AA13" t="str">
+        <v>Programme +21%: 12 wks tender + 5 float for a 400 m² lab. Cost OK.</v>
       </c>
     </row>
     <row r="14">
@@ -1517,37 +1558,40 @@
         <v>-25</v>
       </c>
       <c r="P14" t="str">
-        <v>45–55</v>
+        <v>40–48</v>
       </c>
       <c r="Q14">
         <v>54</v>
       </c>
       <c r="R14" t="str">
-        <v>100–120</v>
+        <v>79–87</v>
       </c>
       <c r="S14">
         <v>101</v>
       </c>
-      <c r="T14" t="str">
+      <c r="T14">
+        <v>22</v>
+      </c>
+      <c r="U14" t="str">
         <v>B</v>
       </c>
-      <c r="U14" t="str">
+      <c r="V14" t="str">
         <v>tight</v>
       </c>
-      <c r="V14" t="str">
+      <c r="W14" t="str">
         <v>Low</v>
       </c>
-      <c r="W14" t="str">
+      <c r="X14" t="str">
         <v>Design and build (single stage)</v>
       </c>
-      <c r="X14" t="str">
+      <c r="Y14" t="str">
         <v>complete</v>
       </c>
-      <c r="Y14" t="str">
+      <c r="Z14" t="str">
         <v>https://www.projento.co.uk/report/b53e6743cb0a492d</v>
       </c>
-      <c r="Z14" t="str">
-        <v>Cost −14% — acceptable. 54 weeks slightly long but fine.</v>
+      <c r="AA14" t="str">
+        <v>Programme +22%: construction 54 wks for a 900 m² GP surgery (40–48), plus 8 float. Cost −14%, acceptable.</v>
       </c>
     </row>
     <row r="15">
@@ -1579,22 +1623,22 @@
         <v>£600k</v>
       </c>
       <c r="J15" t="str">
-        <v>£450k–£630k</v>
+        <v>£360k–£540k</v>
       </c>
       <c r="K15" t="str">
         <v>£296k</v>
       </c>
       <c r="L15">
-        <v>-45</v>
+        <v>-34</v>
       </c>
       <c r="M15" t="str">
-        <v>£680k–£950k</v>
+        <v>£540k–£810k</v>
       </c>
       <c r="N15" t="str">
         <v>£343k–£575k</v>
       </c>
       <c r="O15">
-        <v>-48</v>
+        <v>-37</v>
       </c>
       <c r="P15" t="str">
         <v>14–20</v>
@@ -1603,31 +1647,34 @@
         <v>17</v>
       </c>
       <c r="R15" t="str">
-        <v>45–60</v>
+        <v>43–47</v>
       </c>
       <c r="S15">
         <v>65</v>
       </c>
-      <c r="T15" t="str">
+      <c r="T15">
+        <v>44</v>
+      </c>
+      <c r="U15" t="str">
         <v>D</v>
       </c>
-      <c r="U15" t="str">
+      <c r="V15" t="str">
         <v>tight</v>
       </c>
-      <c r="V15" t="str">
+      <c r="W15" t="str">
         <v>High</v>
       </c>
-      <c r="W15" t="str">
+      <c r="X15" t="str">
         <v>Traditional</v>
       </c>
-      <c r="X15" t="str">
+      <c r="Y15" t="str">
         <v>complete</v>
       </c>
-      <c r="Y15" t="str">
+      <c r="Z15" t="str">
         <v>https://www.projento.co.uk/report/302d0a789a264395</v>
       </c>
-      <c r="Z15" t="str">
-        <v>Cost about 45% below me (£987/m²) for a clinic fit-out with full services — check fit-out healthcare rates.</v>
+      <c r="AA15" t="str">
+        <v>Programme +44%: 12 wks tender for a £300k fit-out (4–6). Cost −34% (£987/m² for a clinic with full services).</v>
       </c>
     </row>
     <row r="16">
@@ -1683,31 +1730,34 @@
         <v>51</v>
       </c>
       <c r="R16" t="str">
-        <v>110–135</v>
+        <v>97–113</v>
       </c>
       <c r="S16">
         <v>96</v>
       </c>
-      <c r="T16" t="str">
+      <c r="T16">
+        <v>-9</v>
+      </c>
+      <c r="U16" t="str">
         <v>D</v>
       </c>
-      <c r="U16" t="str">
+      <c r="V16" t="str">
         <v>tight</v>
       </c>
-      <c r="V16" t="str">
+      <c r="W16" t="str">
         <v>High</v>
       </c>
-      <c r="W16" t="str">
+      <c r="X16" t="str">
         <v>Two-stage (PCSA)</v>
       </c>
-      <c r="X16" t="str">
+      <c r="Y16" t="str">
         <v>complete</v>
       </c>
-      <c r="Y16" t="str">
+      <c r="Z16" t="str">
         <v>https://www.projento.co.uk/report/5ebc54177cb84070</v>
       </c>
-      <c r="Z16" t="str">
-        <v>OK on cost. Range is wide (£6.6m–£11.2m, grade D). No change.</v>
+      <c r="AA16" t="str">
+        <v>Programme OK. Cost OK (wide range, grade D).</v>
       </c>
     </row>
     <row r="17">
@@ -1757,37 +1807,40 @@
         <v>-14</v>
       </c>
       <c r="P17" t="str">
-        <v>6–8</v>
+        <v>5–7</v>
       </c>
       <c r="Q17">
         <v>5</v>
       </c>
       <c r="R17" t="str">
-        <v>14–20</v>
+        <v>12–14</v>
       </c>
       <c r="S17">
         <v>19</v>
       </c>
-      <c r="T17" t="str">
+      <c r="T17">
+        <v>46</v>
+      </c>
+      <c r="U17" t="str">
         <v>B</v>
       </c>
-      <c r="U17" t="str">
+      <c r="V17" t="str">
         <v>tight</v>
       </c>
-      <c r="V17" t="str">
+      <c r="W17" t="str">
         <v>Medium</v>
       </c>
-      <c r="W17" t="str">
+      <c r="X17" t="str">
         <v>Traditional</v>
       </c>
-      <c r="X17" t="str">
+      <c r="Y17" t="str">
         <v>complete</v>
       </c>
-      <c r="Y17" t="str">
+      <c r="Z17" t="str">
         <v>https://www.projento.co.uk/report/a7947cf88d5d4d69</v>
       </c>
-      <c r="Z17" t="str">
-        <v>OK on cost and weeks. No change.</v>
+      <c r="AA17" t="str">
+        <v>Programme +46% (19 vs 12–14 wks): misses the 30 Apr opening date. Cost OK.</v>
       </c>
     </row>
     <row r="18">
@@ -1819,55 +1872,58 @@
         <v>—</v>
       </c>
       <c r="J18" t="str">
-        <v>£2,300k–£3,200k</v>
+        <v>£2,000k–£2,900k</v>
       </c>
       <c r="K18" t="str">
         <v>£1,768k</v>
       </c>
       <c r="L18">
-        <v>-36</v>
+        <v>-28</v>
       </c>
       <c r="M18" t="str">
-        <v>£2,900k–£4,100k</v>
+        <v>£2,500k–£3,600k</v>
       </c>
       <c r="N18" t="str">
         <v>£2,186k–£3,214k</v>
       </c>
       <c r="O18">
-        <v>-26</v>
+        <v>-16</v>
       </c>
       <c r="P18" t="str">
-        <v>36–46</v>
+        <v>40–48</v>
       </c>
       <c r="Q18">
         <v>39</v>
       </c>
       <c r="R18" t="str">
-        <v>85–105</v>
+        <v>87–95</v>
       </c>
       <c r="S18">
         <v>106</v>
       </c>
-      <c r="T18" t="str">
+      <c r="T18">
+        <v>16</v>
+      </c>
+      <c r="U18" t="str">
         <v>C</v>
       </c>
-      <c r="U18" t="str">
+      <c r="V18" t="str">
         <v>none</v>
       </c>
-      <c r="V18" t="str">
+      <c r="W18" t="str">
         <v>High</v>
       </c>
-      <c r="W18" t="str">
+      <c r="X18" t="str">
         <v>Two-stage (PCSA)</v>
       </c>
-      <c r="X18" t="str">
+      <c r="Y18" t="str">
         <v>complete</v>
       </c>
-      <c r="Y18" t="str">
+      <c r="Z18" t="str">
         <v>https://www.projento.co.uk/report/82bfb43318864e66</v>
       </c>
-      <c r="Z18" t="str">
-        <v>Cost about 35% below me (£982/m²) for a full-services store refurb with lift and repairs — check refurb rates.</v>
+      <c r="AA18" t="str">
+        <v>Programme +16% (float 8, gates 6). Cost −28% vs revised (£982/m²).</v>
       </c>
     </row>
     <row r="19">
@@ -1899,22 +1955,22 @@
         <v>£250k</v>
       </c>
       <c r="J19" t="str">
-        <v>£100k–£170k</v>
+        <v>£110k–£190k</v>
       </c>
       <c r="K19" t="str">
         <v>£216k</v>
       </c>
       <c r="L19">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="M19" t="str">
-        <v>£120k–£210k</v>
+        <v>£130k–£230k</v>
       </c>
       <c r="N19" t="str">
         <v>£254k–£340k</v>
       </c>
       <c r="O19">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="P19" t="str">
         <v>6–10</v>
@@ -1923,31 +1979,34 @@
         <v>6</v>
       </c>
       <c r="R19" t="str">
-        <v>20–30</v>
+        <v>22–28</v>
       </c>
       <c r="S19">
         <v>41</v>
       </c>
-      <c r="T19" t="str">
+      <c r="T19">
+        <v>64</v>
+      </c>
+      <c r="U19" t="str">
         <v>B</v>
       </c>
-      <c r="U19" t="str">
+      <c r="V19" t="str">
         <v>insufficient</v>
       </c>
-      <c r="V19" t="str">
+      <c r="W19" t="str">
         <v>Low</v>
       </c>
-      <c r="W19" t="str">
+      <c r="X19" t="str">
         <v>Traditional</v>
       </c>
-      <c r="X19" t="str">
+      <c r="Y19" t="str">
         <v>complete</v>
       </c>
-      <c r="Y19" t="str">
+      <c r="Z19" t="str">
         <v>https://www.projento.co.uk/report/f0408cc053774e23</v>
       </c>
-      <c r="Z19" t="str">
-        <v>Cost about 60% above me (£144/m²) for a single-storey shed demolition; 41-week whole programme is long for a prior-approval demolition.</v>
+      <c r="AA19" t="str">
+        <v>Programme +64%: 14 wks design, 4 gates and 12 wks tender for a £200k demolition. Cost +40% (£144/m²).</v>
       </c>
     </row>
     <row r="20">
@@ -1997,37 +2056,40 @@
         <v>146</v>
       </c>
       <c r="P20" t="str">
-        <v>30–38</v>
+        <v>28–35</v>
       </c>
       <c r="Q20">
         <v>60</v>
       </c>
       <c r="R20" t="str">
-        <v>70–85</v>
+        <v>63–70</v>
       </c>
       <c r="S20">
         <v>122</v>
       </c>
-      <c r="T20" t="str">
+      <c r="T20">
+        <v>83</v>
+      </c>
+      <c r="U20" t="str">
         <v>B</v>
       </c>
-      <c r="U20" t="str">
+      <c r="V20" t="str">
         <v>insufficient</v>
       </c>
-      <c r="V20" t="str">
+      <c r="W20" t="str">
         <v>Low</v>
       </c>
-      <c r="W20" t="str">
+      <c r="X20" t="str">
         <v>Traditional</v>
       </c>
-      <c r="X20" t="str">
+      <c r="Y20" t="str">
         <v>complete</v>
       </c>
-      <c r="Y20" t="str">
+      <c r="Z20" t="str">
         <v>https://www.projento.co.uk/report/e81f15db83864097</v>
       </c>
-      <c r="Z20" t="str">
-        <v>Cost about 2× my estimate (£2,180/m²) — the warehouse shell is still priced like a normal building. Biggest open issue.</v>
+      <c r="AA20" t="str">
+        <v>Programme +83%: 34 wks design and 60 wks construction for a 4,000 m² shed (28–35). Cost ~2× (£2,180/m²): shed shell priced as a normal building.</v>
       </c>
     </row>
     <row r="21">
@@ -2059,22 +2121,22 @@
         <v>—</v>
       </c>
       <c r="J21" t="str">
-        <v>£900k–£1,200k</v>
+        <v>£1,040k–£1,360k</v>
       </c>
       <c r="K21" t="str">
         <v>£1,957k</v>
       </c>
       <c r="L21">
-        <v>86</v>
+        <v>63</v>
       </c>
       <c r="M21" t="str">
-        <v>£1,050k–£1,450k</v>
+        <v>£1,250k–£1,630k</v>
       </c>
       <c r="N21" t="str">
         <v>£2,252k–£3,802k</v>
       </c>
       <c r="O21">
-        <v>125</v>
+        <v>96</v>
       </c>
       <c r="P21" t="str">
         <v>20–26</v>
@@ -2083,31 +2145,34 @@
         <v>32</v>
       </c>
       <c r="R21" t="str">
-        <v>60–75</v>
+        <v>55–61</v>
       </c>
       <c r="S21">
         <v>87</v>
       </c>
-      <c r="T21" t="str">
+      <c r="T21">
+        <v>50</v>
+      </c>
+      <c r="U21" t="str">
         <v>D</v>
       </c>
-      <c r="U21" t="str">
+      <c r="V21" t="str">
         <v>none</v>
       </c>
-      <c r="V21" t="str">
+      <c r="W21" t="str">
         <v>High</v>
       </c>
-      <c r="W21" t="str">
+      <c r="X21" t="str">
         <v>Design and build (single stage)</v>
       </c>
-      <c r="X21" t="str">
+      <c r="Y21" t="str">
         <v>complete</v>
       </c>
-      <c r="Y21" t="str">
+      <c r="Z21" t="str">
         <v>https://www.projento.co.uk/report/07d501ccdd464518</v>
       </c>
-      <c r="Z21" t="str">
-        <v>Cost about 85% above me (£2,446/m²) for a production shed extension — same shell issue as IND-1.</v>
+      <c r="AA21" t="str">
+        <v>Programme +50%: 28 wks design + 12 tender for an 800 m² shed extension. Cost +60% vs revised: same shell issue.</v>
       </c>
     </row>
     <row r="22">
@@ -2157,37 +2222,40 @@
         <v>11</v>
       </c>
       <c r="P22" t="str">
-        <v>12–18</v>
+        <v>12–16</v>
       </c>
       <c r="Q22">
         <v>26</v>
       </c>
       <c r="R22" t="str">
-        <v>45–60</v>
+        <v>40–46</v>
       </c>
       <c r="S22">
         <v>75</v>
       </c>
-      <c r="T22" t="str">
+      <c r="T22">
+        <v>74</v>
+      </c>
+      <c r="U22" t="str">
         <v>B</v>
       </c>
-      <c r="U22" t="str">
+      <c r="V22" t="str">
         <v>tight</v>
       </c>
-      <c r="V22" t="str">
+      <c r="W22" t="str">
         <v>Low</v>
       </c>
-      <c r="W22" t="str">
+      <c r="X22" t="str">
         <v>Traditional</v>
       </c>
-      <c r="X22" t="str">
+      <c r="Y22" t="str">
         <v>complete</v>
       </c>
-      <c r="Y22" t="str">
+      <c r="Z22" t="str">
         <v>https://www.projento.co.uk/report/d984edd9e0ba4d17</v>
       </c>
-      <c r="Z22" t="str">
-        <v>OK on cost. 26 weeks on site for a yard looks long (I expected 12–18).</v>
+      <c r="AA22" t="str">
+        <v>Programme +74%: 24 wks design, 12 tender and 26 wks on site for a yard (12–16). Cost OK.</v>
       </c>
     </row>
     <row r="23">
@@ -2237,37 +2305,40 @@
         <v>47</v>
       </c>
       <c r="P23" t="str">
-        <v>10–14</v>
+        <v>12–14</v>
       </c>
       <c r="Q23">
         <v>8</v>
       </c>
       <c r="R23" t="str">
-        <v>40–55</v>
+        <v>38–42</v>
       </c>
       <c r="S23">
         <v>45</v>
       </c>
-      <c r="T23" t="str">
+      <c r="T23">
+        <v>13</v>
+      </c>
+      <c r="U23" t="str">
         <v>C</v>
       </c>
-      <c r="U23" t="str">
+      <c r="V23" t="str">
         <v>insufficient</v>
       </c>
-      <c r="V23" t="str">
+      <c r="W23" t="str">
         <v>Medium</v>
       </c>
-      <c r="W23" t="str">
+      <c r="X23" t="str">
         <v>Traditional</v>
       </c>
-      <c r="X23" t="str">
+      <c r="Y23" t="str">
         <v>complete</v>
       </c>
-      <c r="Y23" t="str">
+      <c r="Z23" t="str">
         <v>https://www.projento.co.uk/report/f2939a7659f74967</v>
       </c>
-      <c r="Z23" t="str">
-        <v>Cost +27% — high-end restaurant, acceptable. 8 weeks on site looks short for a listed building with a new kitchen (I expected 10–14).</v>
+      <c r="AA23" t="str">
+        <v>Programme OK total, but construction 8 wks short for a listed restaurant with a new kitchen (12–14). Cost +27%, high-end — acceptable.</v>
       </c>
     </row>
     <row r="24">
@@ -2299,22 +2370,22 @@
         <v>£3,500k</v>
       </c>
       <c r="J24" t="str">
-        <v>£2,100k–£3,000k</v>
+        <v>£1,800k–£2,700k</v>
       </c>
       <c r="K24" t="str">
         <v>£1,891k</v>
       </c>
       <c r="L24">
-        <v>-26</v>
+        <v>-16</v>
       </c>
       <c r="M24" t="str">
-        <v>£2,600k–£3,750k</v>
+        <v>£2,250k–£3,400k</v>
       </c>
       <c r="N24" t="str">
         <v>£1,952k–£3,294k</v>
       </c>
       <c r="O24">
-        <v>-23</v>
+        <v>-14</v>
       </c>
       <c r="P24" t="str">
         <v>30–40</v>
@@ -2323,31 +2394,34 @@
         <v>31</v>
       </c>
       <c r="R24" t="str">
-        <v>50–65</v>
+        <v>48–54</v>
       </c>
       <c r="S24">
         <v>63</v>
       </c>
-      <c r="T24" t="str">
+      <c r="T24">
+        <v>24</v>
+      </c>
+      <c r="U24" t="str">
         <v>D</v>
       </c>
-      <c r="U24" t="str">
+      <c r="V24" t="str">
         <v>sufficient</v>
       </c>
-      <c r="V24" t="str">
+      <c r="W24" t="str">
         <v>Low</v>
       </c>
-      <c r="W24" t="str">
+      <c r="X24" t="str">
         <v>Two-stage (PCSA)</v>
       </c>
-      <c r="X24" t="str">
+      <c r="Y24" t="str">
         <v>complete</v>
       </c>
-      <c r="Y24" t="str">
+      <c r="Z24" t="str">
         <v>https://www.projento.co.uk/report/7f920b5676b146d6</v>
       </c>
-      <c r="Z24" t="str">
-        <v>Cost about 25% below me (£630/m²) for 90 bedrooms with en-suites. 3 phases handled (31 weeks).</v>
+      <c r="AA24" t="str">
+        <v>Programme +24%: 12 wks tender + float. Cost OK vs revised.</v>
       </c>
     </row>
     <row r="25">
@@ -2397,37 +2471,40 @@
         <v>-6</v>
       </c>
       <c r="P25" t="str">
-        <v>60–72</v>
+        <v>55–65</v>
       </c>
       <c r="Q25">
         <v>54</v>
       </c>
       <c r="R25" t="str">
-        <v>110–130</v>
+        <v>102–112</v>
       </c>
       <c r="S25">
         <v>117</v>
       </c>
-      <c r="T25" t="str">
+      <c r="T25">
+        <v>9</v>
+      </c>
+      <c r="U25" t="str">
         <v>B</v>
       </c>
-      <c r="U25" t="str">
+      <c r="V25" t="str">
         <v>tight</v>
       </c>
-      <c r="V25" t="str">
+      <c r="W25" t="str">
         <v>Low</v>
       </c>
-      <c r="W25" t="str">
+      <c r="X25" t="str">
         <v>Traditional</v>
       </c>
-      <c r="X25" t="str">
+      <c r="Y25" t="str">
         <v>complete</v>
       </c>
-      <c r="Y25" t="str">
+      <c r="Z25" t="str">
         <v>https://www.projento.co.uk/report/99a049031ae54fd3</v>
       </c>
-      <c r="Z25" t="str">
-        <v>OK on cost (£3,145/m²) and weeks. No change.</v>
+      <c r="AA25" t="str">
+        <v>Programme OK. Cost OK.</v>
       </c>
     </row>
     <row r="26">
@@ -2477,37 +2554,40 @@
         <v>-13</v>
       </c>
       <c r="P26" t="str">
-        <v>40–50</v>
+        <v>40–48</v>
       </c>
       <c r="Q26">
         <v>20</v>
       </c>
       <c r="R26" t="str">
-        <v>90–115</v>
+        <v>83–91</v>
       </c>
       <c r="S26">
         <v>80</v>
       </c>
-      <c r="T26" t="str">
+      <c r="T26">
+        <v>-8</v>
+      </c>
+      <c r="U26" t="str">
         <v>D</v>
       </c>
-      <c r="U26" t="str">
+      <c r="V26" t="str">
         <v>tight</v>
       </c>
-      <c r="V26" t="str">
+      <c r="W26" t="str">
         <v>High</v>
       </c>
-      <c r="W26" t="str">
+      <c r="X26" t="str">
         <v>Traditional</v>
       </c>
-      <c r="X26" t="str">
+      <c r="Y26" t="str">
         <v>complete</v>
       </c>
-      <c r="Y26" t="str">
+      <c r="Z26" t="str">
         <v>https://www.projento.co.uk/report/87fc3d627a394e24</v>
       </c>
-      <c r="Z26" t="str">
-        <v>Cost −20%. 20 weeks on site for a 1,400 m² conversion with a lift looks short (I expected 40–50).</v>
+      <c r="AA26" t="str">
+        <v>Programme OK total but construction 20 wks too short for a 1,400 m² conversion with a lift (40–48). Cost −20% vs mine.</v>
       </c>
     </row>
     <row r="27">
@@ -2557,37 +2637,40 @@
         <v>15</v>
       </c>
       <c r="P27" t="str">
-        <v>60–70</v>
+        <v>55–65</v>
       </c>
       <c r="Q27">
         <v>80</v>
       </c>
       <c r="R27" t="str">
-        <v>95–115</v>
+        <v>82–92</v>
       </c>
       <c r="S27">
         <v>122</v>
       </c>
-      <c r="T27" t="str">
+      <c r="T27">
+        <v>40</v>
+      </c>
+      <c r="U27" t="str">
         <v>C</v>
       </c>
-      <c r="U27" t="str">
+      <c r="V27" t="str">
         <v>insufficient</v>
       </c>
-      <c r="V27" t="str">
+      <c r="W27" t="str">
         <v>Low</v>
       </c>
-      <c r="W27" t="str">
+      <c r="X27" t="str">
         <v>Design and build (single stage)</v>
       </c>
-      <c r="X27" t="str">
+      <c r="Y27" t="str">
         <v>complete</v>
       </c>
-      <c r="Y27" t="str">
+      <c r="Z27" t="str">
         <v>https://www.projento.co.uk/report/766c6ea9ed054088</v>
       </c>
-      <c r="Z27" t="str">
-        <v>Cost +16% and 80 weeks vs my 60–70 — slightly high on both.</v>
+      <c r="AA27" t="str">
+        <v>Programme +40%: construction 80 wks for a 3,200 m² 4-storey block (55–65). Cost +16%.</v>
       </c>
     </row>
     <row r="28">
@@ -2637,37 +2720,40 @@
         <v>1</v>
       </c>
       <c r="P28" t="str">
-        <v>12–18</v>
+        <v>10–16</v>
       </c>
       <c r="Q28">
         <v>10</v>
       </c>
       <c r="R28" t="str">
-        <v>35–50</v>
+        <v>33–39</v>
       </c>
       <c r="S28">
         <v>56</v>
       </c>
-      <c r="T28" t="str">
+      <c r="T28">
+        <v>56</v>
+      </c>
+      <c r="U28" t="str">
         <v>C</v>
       </c>
-      <c r="U28" t="str">
+      <c r="V28" t="str">
         <v>none</v>
       </c>
-      <c r="V28" t="str">
+      <c r="W28" t="str">
         <v>High</v>
       </c>
-      <c r="W28" t="str">
+      <c r="X28" t="str">
         <v>Traditional</v>
       </c>
-      <c r="X28" t="str">
+      <c r="Y28" t="str">
         <v>complete</v>
       </c>
-      <c r="Y28" t="str">
+      <c r="Z28" t="str">
         <v>https://www.projento.co.uk/report/82bdb8fcd9b240cb</v>
       </c>
-      <c r="Z28" t="str">
-        <v>OK on cost and weeks. No change.</v>
+      <c r="AA28" t="str">
+        <v>Programme +56%: 29 wks of design stages for a demolition. Cost OK.</v>
       </c>
     </row>
     <row r="29">
@@ -2717,37 +2803,40 @@
         <v>-7</v>
       </c>
       <c r="P29" t="str">
-        <v>30–38</v>
+        <v>30–36</v>
       </c>
       <c r="Q29">
         <v>23</v>
       </c>
       <c r="R29" t="str">
-        <v>75–95</v>
+        <v>65–71</v>
       </c>
       <c r="S29">
         <v>74</v>
       </c>
-      <c r="T29" t="str">
+      <c r="T29">
+        <v>9</v>
+      </c>
+      <c r="U29" t="str">
         <v>C</v>
       </c>
-      <c r="U29" t="str">
+      <c r="V29" t="str">
         <v>insufficient</v>
       </c>
-      <c r="V29" t="str">
+      <c r="W29" t="str">
         <v>Medium</v>
       </c>
-      <c r="W29" t="str">
+      <c r="X29" t="str">
         <v>Traditional</v>
       </c>
-      <c r="X29" t="str">
+      <c r="Y29" t="str">
         <v>complete</v>
       </c>
-      <c r="Y29" t="str">
+      <c r="Z29" t="str">
         <v>https://www.projento.co.uk/report/73e49cd5107e41f7</v>
       </c>
-      <c r="Z29" t="str">
-        <v>OK on cost. 23 weeks looks short for refurb plus a hall extension (I expected 30–38).</v>
+      <c r="AA29" t="str">
+        <v>Programme OK total; construction 23 wks short for refurb + hall extension (30–36). Cost OK.</v>
       </c>
     </row>
     <row r="30">
@@ -2779,55 +2868,58 @@
         <v>£700k</v>
       </c>
       <c r="J30" t="str">
-        <v>£540k–£750k</v>
+        <v>£450k–£660k</v>
       </c>
       <c r="K30" t="str">
         <v>£307k</v>
       </c>
       <c r="L30">
-        <v>-52</v>
+        <v>-45</v>
       </c>
       <c r="M30" t="str">
-        <v>£800k–£1,100k</v>
+        <v>£680k–£990k</v>
       </c>
       <c r="N30" t="str">
         <v>£380k–£561k</v>
       </c>
       <c r="O30">
-        <v>-53</v>
+        <v>-46</v>
       </c>
       <c r="P30" t="str">
-        <v>20–26</v>
+        <v>18–24</v>
       </c>
       <c r="Q30">
         <v>13</v>
       </c>
       <c r="R30" t="str">
-        <v>70–90</v>
+        <v>56–62</v>
       </c>
       <c r="S30">
         <v>66</v>
       </c>
-      <c r="T30" t="str">
+      <c r="T30">
+        <v>12</v>
+      </c>
+      <c r="U30" t="str">
         <v>C</v>
       </c>
-      <c r="U30" t="str">
+      <c r="V30" t="str">
         <v>sufficient</v>
       </c>
-      <c r="V30" t="str">
+      <c r="W30" t="str">
         <v>High</v>
       </c>
-      <c r="W30" t="str">
+      <c r="X30" t="str">
         <v>Traditional</v>
       </c>
-      <c r="X30" t="str">
+      <c r="Y30" t="str">
         <v>complete</v>
       </c>
-      <c r="Y30" t="str">
+      <c r="Z30" t="str">
         <v>https://www.projento.co.uk/report/80d9e5e3d1d540a5</v>
       </c>
-      <c r="Z30" t="str">
-        <v>Cost about 50% below me (£1,023/m²) for a listed church hall with new services, repairs and damp work.</v>
+      <c r="AA30" t="str">
+        <v>Programme OK total; construction 13 wks short for a listed hall (18–24). Cost −45% (£1,023/m²).</v>
       </c>
     </row>
     <row r="31">
@@ -2877,43 +2969,128 @@
         <v>-12</v>
       </c>
       <c r="P31" t="str">
-        <v>10–14</v>
+        <v>10–12</v>
       </c>
       <c r="Q31">
         <v>7</v>
       </c>
       <c r="R31" t="str">
-        <v>35–50</v>
+        <v>33–40</v>
       </c>
       <c r="S31">
         <v>46</v>
       </c>
-      <c r="T31" t="str">
+      <c r="T31">
+        <v>26</v>
+      </c>
+      <c r="U31" t="str">
         <v>B</v>
       </c>
-      <c r="U31" t="str">
+      <c r="V31" t="str">
         <v>sufficient</v>
       </c>
-      <c r="V31" t="str">
+      <c r="W31" t="str">
         <v>Low</v>
       </c>
-      <c r="W31" t="str">
+      <c r="X31" t="str">
         <v>Traditional</v>
       </c>
-      <c r="X31" t="str">
+      <c r="Y31" t="str">
         <v>complete</v>
       </c>
-      <c r="Y31" t="str">
+      <c r="Z31" t="str">
         <v>https://www.projento.co.uk/report/cdea78a268874ac2</v>
       </c>
-      <c r="Z31" t="str">
-        <v>OK on cost. 7 weeks on site looks short for a 500 m² library (I expected 10–14).</v>
+      <c r="AA31" t="str">
+        <v>Programme +26%: 12 wks tender for a £300k fit-out; construction 7 wks short (10–12). Cost OK.</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z31"/>
+  <autoFilter ref="A1:AA31"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA31"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C6"/>
+  <cols>
+    <col min="1" max="1" width="34.83203125" customWidth="1"/>
+    <col min="2" max="2" width="70.83203125" customWidth="1"/>
+    <col min="3" max="3" width="60.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Cause</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Evidence (30 reports)</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Suggested fix (workbook, for your decision)</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>1. Programme float added on top</v>
+      </c>
+      <c r="B2" t="str">
+        <v>+1 wk per 13 wks (PROG-FLOAT) on every report: 2–12 wks, average 6. The stage durations are already range mid-points.</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Show float as a risk allowance, not in the headline; or halve it (1 wk per 26).</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>2. Tender 12 weeks regardless of size</v>
+      </c>
+      <c r="B3" t="str">
+        <v>22 of 30 get 12 wks, incl. £200k demolition, £300k fit-outs and a car park.</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Tender by value: under £500k 4–6 wks, £0.5–2m 8, over £2m 10–12 (TN1 bands).</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>3. Client gateway after every stage</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2 wks after each design stage: 2–6 wks per report, average 4.</v>
+      </c>
+      <c r="C4" t="str">
+        <v>1 wk on small jobs, or only after Stage 2 and Stage 4.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>4. Full design stages on simple jobs</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Demolition MIX-3 29 wks design, RET-3 14; yard IND-3 24; car park RES-3 20; warehouse IND-1 34.</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Shorter design rows for Demolition, External works and sheds (one combined design stage).</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>5. Construction too long on large/simple, too short on small refurbs</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Too long: warehouse 60 (28–35), 4-storey mixed 80 (55–65), GP 54 (40–48), Cat A 23 (12–16), yard 26. Too short: conversion 20 (40–48), classroom ext 15, library 7, church hall 13.</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Shed row for industrial; review CN rows for S5–S6 new build; raise small refurb / conversion rows.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>